<commit_message>
Updates from weekend and minor fixes
</commit_message>
<xml_diff>
--- a/public/Data/HEMANPUNTERS.xlsx
+++ b/public/Data/HEMANPUNTERS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bturnor\Repos\seeMore\public\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEB900C8-65A0-49F6-8575-5F9E5CDEF57C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BAEF0170-E0A5-46D2-B033-19D78F6C50F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="6" activeTab="8" xr2:uid="{525E8989-1938-4309-A4CF-8F1D15E362FB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="8" activeTab="8" xr2:uid="{525E8989-1938-4309-A4CF-8F1D15E362FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Punters club" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="191">
   <si>
     <t>HE_MAN PUNTERS 2019</t>
   </si>
@@ -612,7 +612,34 @@
     <t>A.BAXTER</t>
   </si>
   <si>
+    <t>Total bet and return for all seasons</t>
+  </si>
+  <si>
+    <t>adam</t>
+  </si>
+  <si>
+    <t>1 leg losses as at 09/03/2026</t>
+  </si>
+  <si>
+    <t>Strikes for 2026 Season at 09/03/2026</t>
+  </si>
+  <si>
     <t>Adam</t>
+  </si>
+  <si>
+    <t>Jamie Elliot needed 2 goals, got 1 goal 1 point</t>
+  </si>
+  <si>
+    <t>Worpel needed 20 or more, got 17</t>
+  </si>
+  <si>
+    <t>Max Verstappen needed to podium finish</t>
+  </si>
+  <si>
+    <t>Wanganeen-Milera needed 25 or more, got 19</t>
+  </si>
+  <si>
+    <t>Wanganeen-Milera Needed 30 or more, got 19</t>
   </si>
 </sst>
 </file>
@@ -790,7 +817,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="33">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -1230,12 +1257,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1358,6 +1409,11 @@
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1416,6 +1472,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4133,7 +4192,7 @@
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" customWidth="1"/>
     <col min="3" max="3" width="20.44140625" customWidth="1"/>
-    <col min="4" max="4" width="39.33203125" customWidth="1"/>
+    <col min="4" max="4" width="41.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -4162,7 +4221,18 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C2" s="59"/>
+      <c r="A2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" s="60">
+        <v>10</v>
+      </c>
+      <c r="C2" s="59">
+        <v>358</v>
+      </c>
+      <c r="D2" t="s">
+        <v>186</v>
+      </c>
       <c r="E2" t="s">
         <v>12</v>
       </c>
@@ -4176,22 +4246,43 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C3" s="59"/>
+      <c r="A3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="60">
+        <v>10</v>
+      </c>
+      <c r="C3" s="59">
+        <v>95</v>
+      </c>
+      <c r="D3" t="s">
+        <v>187</v>
+      </c>
       <c r="E3" t="s">
         <v>94</v>
       </c>
-      <c r="F3" t="str">
+      <c r="F3">
         <f t="shared" si="0"/>
-        <v/>
+        <v>95</v>
       </c>
       <c r="G3">
         <f>COUNTIF(A1:A81, E3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B4" s="60"/>
-      <c r="C4" s="59"/>
+      <c r="A4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B4" s="60">
+        <v>10</v>
+      </c>
+      <c r="C4" s="59">
+        <v>61.8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>188</v>
+      </c>
       <c r="E4" t="s">
         <v>95</v>
       </c>
@@ -4200,13 +4291,23 @@
         <v/>
       </c>
       <c r="G4">
-        <f t="shared" ref="G4" si="1">COUNTIF(A4:A84, E4)</f>
+        <f>COUNTIF(A2:A84, E4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
+      <c r="A5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" s="59">
+        <v>10</v>
+      </c>
+      <c r="C5" s="59">
+        <v>95</v>
+      </c>
+      <c r="D5" t="s">
+        <v>189</v>
+      </c>
       <c r="E5" t="s">
         <v>93</v>
       </c>
@@ -4215,23 +4316,33 @@
         <v/>
       </c>
       <c r="G5">
-        <f t="shared" ref="G5" si="2">COUNTIF(A4:A84, E5)</f>
+        <f>COUNTIF(A2:A84, E5)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B6" s="59"/>
-      <c r="C6" s="59"/>
+      <c r="A6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="59">
+        <v>10</v>
+      </c>
+      <c r="C6" s="59">
+        <v>97.5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>190</v>
+      </c>
       <c r="E6" t="s">
         <v>97</v>
       </c>
-      <c r="F6" t="str">
+      <c r="F6">
         <f t="shared" si="0"/>
-        <v/>
+        <v>95</v>
       </c>
       <c r="G6">
-        <f t="shared" ref="G6" si="3">COUNTIF(A4:A84, E6)</f>
-        <v>0</v>
+        <f>COUNTIF(A2:A84, E6)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -4245,7 +4356,7 @@
         <v/>
       </c>
       <c r="G7">
-        <f t="shared" ref="G7" si="4">COUNTIF(A7:A87, E7)</f>
+        <f>COUNTIF(A2:A87, E7)</f>
         <v>0</v>
       </c>
     </row>
@@ -4255,13 +4366,13 @@
       <c r="E8" t="s">
         <v>89</v>
       </c>
-      <c r="F8" t="str">
+      <c r="F8">
         <f t="shared" si="0"/>
-        <v/>
+        <v>97.5</v>
       </c>
       <c r="G8">
-        <f t="shared" ref="G8" si="5">COUNTIF(A7:A87, E8)</f>
-        <v>0</v>
+        <f>COUNTIF(A2:A87, E8)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -4275,7 +4386,7 @@
         <v/>
       </c>
       <c r="G9">
-        <f t="shared" ref="G9" si="6">COUNTIF(A7:A87, E9)</f>
+        <f>COUNTIF(A2:A87, E9)</f>
         <v>0</v>
       </c>
     </row>
@@ -4290,7 +4401,7 @@
         <v/>
       </c>
       <c r="G10">
-        <f t="shared" ref="G10" si="7">COUNTIF(A10:A90, E10)</f>
+        <f>COUNTIF(A2:A90, E10)</f>
         <v>0</v>
       </c>
     </row>
@@ -4300,13 +4411,13 @@
       <c r="E11" t="s">
         <v>121</v>
       </c>
-      <c r="F11" t="str">
+      <c r="F11">
         <f t="shared" si="0"/>
-        <v/>
+        <v>358</v>
       </c>
       <c r="G11">
-        <f>COUNTIF(A10:A90, E11)</f>
-        <v>0</v>
+        <f>COUNTIF(A2:A90, E11)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -4320,7 +4431,7 @@
         <v/>
       </c>
       <c r="G12">
-        <f t="shared" ref="G12" si="8">COUNTIF(A10:A90, E12)</f>
+        <f>COUNTIF(A2:A90, E12)</f>
         <v>0</v>
       </c>
     </row>
@@ -4328,15 +4439,15 @@
       <c r="B13" s="60"/>
       <c r="C13" s="59"/>
       <c r="E13" t="s">
-        <v>181</v>
-      </c>
-      <c r="F13" t="str">
+        <v>185</v>
+      </c>
+      <c r="F13">
         <f t="shared" si="0"/>
-        <v/>
+        <v>61.8</v>
       </c>
       <c r="G13">
         <f>COUNTIF(A2:A100, E13)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -4344,7 +4455,11 @@
       <c r="C14" s="59"/>
       <c r="F14" s="61">
         <f>SUM(F1:F13)</f>
-        <v>0</v>
+        <v>707.3</v>
+      </c>
+      <c r="G14">
+        <f>SUM(G1:G13)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -4519,50 +4634,50 @@
   <sheetData>
     <row r="1" spans="2:27" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:27" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C2" s="62" t="s">
+      <c r="C2" s="67" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62" t="s">
+      <c r="D2" s="67"/>
+      <c r="E2" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62" t="s">
+      <c r="F2" s="67"/>
+      <c r="G2" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62" t="s">
+      <c r="H2" s="67"/>
+      <c r="I2" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62" t="s">
+      <c r="J2" s="67"/>
+      <c r="K2" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="62"/>
-      <c r="M2" s="62" t="s">
+      <c r="L2" s="67"/>
+      <c r="M2" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62" t="s">
+      <c r="N2" s="67"/>
+      <c r="O2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62" t="s">
-        <v>25</v>
-      </c>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62" t="s">
+      <c r="P2" s="67"/>
+      <c r="Q2" s="67" t="s">
+        <v>25</v>
+      </c>
+      <c r="R2" s="67"/>
+      <c r="S2" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62" t="s">
+      <c r="T2" s="67"/>
+      <c r="U2" s="67" t="s">
         <v>27</v>
       </c>
-      <c r="V2" s="69"/>
-      <c r="W2" s="68" t="s">
+      <c r="V2" s="74"/>
+      <c r="W2" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="X2" s="62"/>
+      <c r="X2" s="67"/>
     </row>
     <row r="3" spans="2:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="32" t="s">
@@ -6123,34 +6238,34 @@
       </c>
     </row>
     <row r="29" spans="2:27" x14ac:dyDescent="0.3">
-      <c r="F29" s="65" t="s">
+      <c r="F29" s="70" t="s">
         <v>56</v>
       </c>
-      <c r="G29" s="66"/>
-      <c r="H29" s="67"/>
-      <c r="I29" s="63">
+      <c r="G29" s="71"/>
+      <c r="H29" s="72"/>
+      <c r="I29" s="68">
         <f>C27+E27+G27+I27+K27+M27+O27+Q27+S27+U27</f>
         <v>2469.42</v>
       </c>
-      <c r="J29" s="64"/>
+      <c r="J29" s="69"/>
     </row>
     <row r="30" spans="2:27" x14ac:dyDescent="0.3">
-      <c r="G30" s="70" t="s">
+      <c r="G30" s="75" t="s">
         <v>57</v>
       </c>
-      <c r="H30" s="70"/>
-      <c r="I30" s="63">
+      <c r="H30" s="75"/>
+      <c r="I30" s="68">
         <f>+D27+F27+H27+J27+L27+N27+P27+R27+T27+V27</f>
         <v>1774.69</v>
       </c>
-      <c r="J30" s="64"/>
+      <c r="J30" s="69"/>
     </row>
     <row r="31" spans="2:27" x14ac:dyDescent="0.3">
-      <c r="I31" s="63">
+      <c r="I31" s="68">
         <f>I30-I29</f>
         <v>-694.73</v>
       </c>
-      <c r="J31" s="64"/>
+      <c r="J31" s="69"/>
     </row>
     <row r="32" spans="2:27" x14ac:dyDescent="0.3">
       <c r="C32" s="1">
@@ -6199,11 +6314,11 @@
       </c>
     </row>
     <row r="34" spans="3:16" x14ac:dyDescent="0.3">
-      <c r="I34" s="64">
+      <c r="I34" s="69">
         <f>I33+I31</f>
         <v>505.27</v>
       </c>
-      <c r="J34" s="64"/>
+      <c r="J34" s="69"/>
     </row>
     <row r="38" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C38" s="1">
@@ -6291,50 +6406,50 @@
   <sheetData>
     <row r="1" spans="2:27" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:27" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C2" s="62" t="s">
+      <c r="C2" s="67" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62" t="s">
+      <c r="D2" s="67"/>
+      <c r="E2" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="62"/>
-      <c r="G2" s="72" t="s">
+      <c r="F2" s="67"/>
+      <c r="G2" s="77" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="68"/>
-      <c r="I2" s="62" t="s">
+      <c r="H2" s="73"/>
+      <c r="I2" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62" t="s">
+      <c r="J2" s="67"/>
+      <c r="K2" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="L2" s="62"/>
-      <c r="M2" s="62" t="s">
-        <v>25</v>
-      </c>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62" t="s">
+      <c r="L2" s="67"/>
+      <c r="M2" s="67" t="s">
+        <v>25</v>
+      </c>
+      <c r="N2" s="67"/>
+      <c r="O2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62" t="s">
+      <c r="P2" s="67"/>
+      <c r="Q2" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62" t="s">
+      <c r="R2" s="67"/>
+      <c r="S2" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62" t="s">
+      <c r="T2" s="67"/>
+      <c r="U2" s="67" t="s">
         <v>27</v>
       </c>
-      <c r="V2" s="69"/>
-      <c r="W2" s="68" t="s">
+      <c r="V2" s="74"/>
+      <c r="W2" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="X2" s="62"/>
+      <c r="X2" s="67"/>
     </row>
     <row r="3" spans="2:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="32" t="s">
@@ -7694,34 +7809,34 @@
       </c>
     </row>
     <row r="29" spans="2:27" x14ac:dyDescent="0.3">
-      <c r="F29" s="65" t="s">
+      <c r="F29" s="70" t="s">
         <v>56</v>
       </c>
-      <c r="G29" s="66"/>
-      <c r="H29" s="67"/>
-      <c r="I29" s="63">
+      <c r="G29" s="71"/>
+      <c r="H29" s="72"/>
+      <c r="I29" s="68">
         <f>C27+E27+G27+I27+K27+M27+O27+Q27+S27+U27</f>
         <v>1788.24</v>
       </c>
-      <c r="J29" s="64"/>
+      <c r="J29" s="69"/>
     </row>
     <row r="30" spans="2:27" x14ac:dyDescent="0.3">
-      <c r="G30" s="70" t="s">
+      <c r="G30" s="75" t="s">
         <v>57</v>
       </c>
-      <c r="H30" s="70"/>
-      <c r="I30" s="63">
+      <c r="H30" s="75"/>
+      <c r="I30" s="68">
         <f>+D27+F27+H27+J27+L27+N27+P27+R27+T27+V27</f>
         <v>2492.1999999999998</v>
       </c>
-      <c r="J30" s="64"/>
+      <c r="J30" s="69"/>
     </row>
     <row r="31" spans="2:27" x14ac:dyDescent="0.3">
-      <c r="I31" s="63">
+      <c r="I31" s="68">
         <f>I30-I29</f>
         <v>703.95999999999981</v>
       </c>
-      <c r="J31" s="64"/>
+      <c r="J31" s="69"/>
     </row>
     <row r="32" spans="2:27" x14ac:dyDescent="0.3">
       <c r="C32" s="36">
@@ -7775,11 +7890,11 @@
         <v>64</v>
       </c>
       <c r="H34" s="42"/>
-      <c r="I34" s="71">
+      <c r="I34" s="76">
         <f>I33+I31</f>
         <v>1303.9599999999998</v>
       </c>
-      <c r="J34" s="71"/>
+      <c r="J34" s="76"/>
       <c r="M34" s="33"/>
     </row>
     <row r="38" spans="3:16" x14ac:dyDescent="0.3">
@@ -7869,54 +7984,54 @@
   <sheetData>
     <row r="1" spans="2:34" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:34" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C2" s="62" t="s">
+      <c r="C2" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62" t="s">
+      <c r="D2" s="67"/>
+      <c r="E2" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62" t="s">
+      <c r="F2" s="67"/>
+      <c r="G2" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62" t="s">
+      <c r="H2" s="67"/>
+      <c r="I2" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62" t="s">
+      <c r="J2" s="67"/>
+      <c r="K2" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="62"/>
-      <c r="M2" s="62" t="s">
+      <c r="L2" s="67"/>
+      <c r="M2" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62" t="s">
+      <c r="N2" s="67"/>
+      <c r="O2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62" t="s">
-        <v>25</v>
-      </c>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62" t="s">
+      <c r="P2" s="67"/>
+      <c r="Q2" s="67" t="s">
+        <v>25</v>
+      </c>
+      <c r="R2" s="67"/>
+      <c r="S2" s="67" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62" t="s">
+      <c r="T2" s="67"/>
+      <c r="U2" s="67" t="s">
         <v>65</v>
       </c>
-      <c r="V2" s="69"/>
-      <c r="W2" s="62" t="s">
+      <c r="V2" s="74"/>
+      <c r="W2" s="67" t="s">
         <v>66</v>
       </c>
-      <c r="X2" s="69"/>
-      <c r="Y2" s="68" t="s">
+      <c r="X2" s="74"/>
+      <c r="Y2" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="Z2" s="62"/>
+      <c r="Z2" s="67"/>
     </row>
     <row r="3" spans="2:34" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="32" t="s">
@@ -9970,34 +10085,34 @@
       </c>
     </row>
     <row r="31" spans="2:30" x14ac:dyDescent="0.3">
-      <c r="F31" s="65" t="s">
+      <c r="F31" s="70" t="s">
         <v>56</v>
       </c>
-      <c r="G31" s="66"/>
-      <c r="H31" s="67"/>
-      <c r="I31" s="63">
+      <c r="G31" s="71"/>
+      <c r="H31" s="72"/>
+      <c r="I31" s="68">
         <f>C29+E29+G29+I29+K29+M29+O29+Q29+S29+U29+W29</f>
         <v>2521.33</v>
       </c>
-      <c r="J31" s="64"/>
+      <c r="J31" s="69"/>
     </row>
     <row r="32" spans="2:30" x14ac:dyDescent="0.3">
-      <c r="G32" s="70" t="s">
+      <c r="G32" s="75" t="s">
         <v>57</v>
       </c>
-      <c r="H32" s="70"/>
-      <c r="I32" s="63">
+      <c r="H32" s="75"/>
+      <c r="I32" s="68">
         <f>+D29+F29+H29+J29+L29+N29+P29+R29+T29+V29+X29</f>
         <v>2997.5899999999997</v>
       </c>
-      <c r="J32" s="64"/>
+      <c r="J32" s="69"/>
     </row>
     <row r="33" spans="3:17" x14ac:dyDescent="0.3">
-      <c r="I33" s="63">
+      <c r="I33" s="68">
         <f>I32-I31</f>
         <v>476.25999999999976</v>
       </c>
-      <c r="J33" s="64"/>
+      <c r="J33" s="69"/>
     </row>
     <row r="34" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C34" s="36">
@@ -10050,11 +10165,11 @@
         <v>64</v>
       </c>
       <c r="H36" s="42"/>
-      <c r="I36" s="71">
+      <c r="I36" s="76">
         <f>I35+I33</f>
         <v>2476.2599999999998</v>
       </c>
-      <c r="J36" s="71"/>
+      <c r="J36" s="76"/>
       <c r="M36" s="33"/>
     </row>
     <row r="40" spans="3:17" x14ac:dyDescent="0.3">
@@ -10145,54 +10260,54 @@
   <sheetData>
     <row r="1" spans="2:34" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:34" ht="18" x14ac:dyDescent="0.35">
-      <c r="C2" s="62" t="s">
+      <c r="C2" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="62"/>
-      <c r="E2" s="72" t="s">
+      <c r="D2" s="67"/>
+      <c r="E2" s="77" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="68"/>
-      <c r="G2" s="62" t="s">
+      <c r="F2" s="73"/>
+      <c r="G2" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62" t="s">
+      <c r="H2" s="67"/>
+      <c r="I2" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62" t="s">
+      <c r="J2" s="67"/>
+      <c r="K2" s="67" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="62"/>
-      <c r="M2" s="72" t="s">
+      <c r="L2" s="67"/>
+      <c r="M2" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="N2" s="68"/>
-      <c r="O2" s="62" t="s">
-        <v>25</v>
-      </c>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62" t="s">
+      <c r="N2" s="73"/>
+      <c r="O2" s="67" t="s">
+        <v>25</v>
+      </c>
+      <c r="P2" s="67"/>
+      <c r="Q2" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62" t="s">
+      <c r="R2" s="67"/>
+      <c r="S2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62" t="s">
+      <c r="T2" s="67"/>
+      <c r="U2" s="67" t="s">
         <v>65</v>
       </c>
-      <c r="V2" s="69"/>
-      <c r="W2" s="62" t="s">
+      <c r="V2" s="74"/>
+      <c r="W2" s="67" t="s">
         <v>66</v>
       </c>
-      <c r="X2" s="69"/>
-      <c r="Y2" s="68" t="s">
+      <c r="X2" s="74"/>
+      <c r="Y2" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="Z2" s="62"/>
+      <c r="Z2" s="67"/>
     </row>
     <row r="3" spans="2:34" x14ac:dyDescent="0.3">
       <c r="B3" s="32" t="s">
@@ -12201,34 +12316,34 @@
       </c>
     </row>
     <row r="31" spans="2:30" x14ac:dyDescent="0.3">
-      <c r="F31" s="65" t="s">
+      <c r="F31" s="70" t="s">
         <v>56</v>
       </c>
-      <c r="G31" s="66"/>
-      <c r="H31" s="67"/>
-      <c r="I31" s="63">
+      <c r="G31" s="71"/>
+      <c r="H31" s="72"/>
+      <c r="I31" s="68">
         <f>C29+E29+G29+I29+K29+M29+O29+Q29+S29+U29+W29</f>
         <v>2462.73</v>
       </c>
-      <c r="J31" s="64"/>
+      <c r="J31" s="69"/>
     </row>
     <row r="32" spans="2:30" x14ac:dyDescent="0.3">
-      <c r="G32" s="70" t="s">
+      <c r="G32" s="75" t="s">
         <v>57</v>
       </c>
-      <c r="H32" s="70"/>
-      <c r="I32" s="63">
+      <c r="H32" s="75"/>
+      <c r="I32" s="68">
         <f>+D29+F29+H29+J29+L29+N29+P29+R29+T29+V29+X29</f>
         <v>1004.25</v>
       </c>
-      <c r="J32" s="64"/>
+      <c r="J32" s="69"/>
     </row>
     <row r="33" spans="3:25" x14ac:dyDescent="0.3">
-      <c r="I33" s="63">
+      <c r="I33" s="68">
         <f>I32-I31</f>
         <v>-1458.48</v>
       </c>
-      <c r="J33" s="64"/>
+      <c r="J33" s="69"/>
       <c r="Y33">
         <f>2167+183+5*10</f>
         <v>2400</v>
@@ -12324,11 +12439,11 @@
         <v>64</v>
       </c>
       <c r="H38" s="42"/>
-      <c r="I38" s="71">
+      <c r="I38" s="76">
         <f>I36+I33+J37</f>
         <v>322.7800000000002</v>
       </c>
-      <c r="J38" s="71"/>
+      <c r="J38" s="76"/>
       <c r="M38" s="33"/>
     </row>
     <row r="40" spans="3:25" x14ac:dyDescent="0.3">
@@ -12650,54 +12765,54 @@
   <sheetData>
     <row r="1" spans="2:34" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:34" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C2" s="62" t="s">
+      <c r="C2" s="67" t="s">
         <v>100</v>
       </c>
-      <c r="D2" s="62"/>
-      <c r="E2" s="72" t="s">
+      <c r="D2" s="67"/>
+      <c r="E2" s="77" t="s">
         <v>101</v>
       </c>
-      <c r="F2" s="68"/>
-      <c r="G2" s="62" t="s">
+      <c r="F2" s="73"/>
+      <c r="G2" s="67" t="s">
         <v>102</v>
       </c>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62" t="s">
+      <c r="H2" s="67"/>
+      <c r="I2" s="67" t="s">
         <v>103</v>
       </c>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62" t="s">
+      <c r="J2" s="67"/>
+      <c r="K2" s="67" t="s">
         <v>104</v>
       </c>
-      <c r="L2" s="62"/>
-      <c r="M2" s="72" t="s">
+      <c r="L2" s="67"/>
+      <c r="M2" s="77" t="s">
         <v>105</v>
       </c>
-      <c r="N2" s="68"/>
-      <c r="O2" s="62" t="s">
+      <c r="N2" s="73"/>
+      <c r="O2" s="67" t="s">
         <v>106</v>
       </c>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62" t="s">
+      <c r="P2" s="67"/>
+      <c r="Q2" s="67" t="s">
         <v>107</v>
       </c>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62" t="s">
+      <c r="R2" s="67"/>
+      <c r="S2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62" t="s">
+      <c r="T2" s="67"/>
+      <c r="U2" s="67" t="s">
         <v>108</v>
       </c>
-      <c r="V2" s="69"/>
-      <c r="W2" s="62" t="s">
+      <c r="V2" s="74"/>
+      <c r="W2" s="67" t="s">
         <v>66</v>
       </c>
-      <c r="X2" s="69"/>
-      <c r="Y2" s="68" t="s">
+      <c r="X2" s="74"/>
+      <c r="Y2" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="Z2" s="62"/>
+      <c r="Z2" s="67"/>
     </row>
     <row r="3" spans="2:34" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="32" t="s">
@@ -14680,34 +14795,34 @@
       </c>
     </row>
     <row r="31" spans="2:30" x14ac:dyDescent="0.3">
-      <c r="F31" s="65" t="s">
+      <c r="F31" s="70" t="s">
         <v>56</v>
       </c>
-      <c r="G31" s="66"/>
-      <c r="H31" s="67"/>
-      <c r="I31" s="63">
+      <c r="G31" s="71"/>
+      <c r="H31" s="72"/>
+      <c r="I31" s="68">
         <f>C29+E29+G29+I29+K29+M29+O29+Q29+S29+U29+W29</f>
         <v>2158</v>
       </c>
-      <c r="J31" s="64"/>
+      <c r="J31" s="69"/>
     </row>
     <row r="32" spans="2:30" x14ac:dyDescent="0.3">
-      <c r="G32" s="70" t="s">
+      <c r="G32" s="75" t="s">
         <v>57</v>
       </c>
-      <c r="H32" s="70"/>
-      <c r="I32" s="63">
+      <c r="H32" s="75"/>
+      <c r="I32" s="68">
         <f>+D29+F29+H29+J29+L29+N29+P29+R29+T29+V29+X29</f>
         <v>709.26</v>
       </c>
-      <c r="J32" s="64"/>
+      <c r="J32" s="69"/>
     </row>
     <row r="33" spans="3:25" x14ac:dyDescent="0.3">
-      <c r="I33" s="63">
+      <c r="I33" s="68">
         <f>I32-I31</f>
         <v>-1448.74</v>
       </c>
-      <c r="J33" s="64"/>
+      <c r="J33" s="69"/>
       <c r="Y33">
         <f>2167+183+5*10</f>
         <v>2400</v>
@@ -14796,11 +14911,11 @@
         <v>64</v>
       </c>
       <c r="H38" s="42"/>
-      <c r="I38" s="71">
+      <c r="I38" s="76">
         <f>I36+I33</f>
         <v>552.84999999999991</v>
       </c>
-      <c r="J38" s="71"/>
+      <c r="J38" s="76"/>
       <c r="M38" s="33"/>
     </row>
     <row r="40" spans="3:25" x14ac:dyDescent="0.3">
@@ -15155,66 +15270,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:38" ht="7.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="W1" s="73"/>
-      <c r="X1" s="74"/>
+      <c r="W1" s="78"/>
+      <c r="X1" s="79"/>
     </row>
     <row r="2" spans="2:38" ht="18" x14ac:dyDescent="0.35">
-      <c r="C2" s="62" t="s">
+      <c r="C2" s="67" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="62"/>
-      <c r="E2" s="72" t="s">
+      <c r="D2" s="67"/>
+      <c r="E2" s="77" t="s">
         <v>101</v>
       </c>
-      <c r="F2" s="68"/>
-      <c r="G2" s="62" t="s">
+      <c r="F2" s="73"/>
+      <c r="G2" s="67" t="s">
         <v>114</v>
       </c>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62" t="s">
+      <c r="H2" s="67"/>
+      <c r="I2" s="67" t="s">
         <v>115</v>
       </c>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62" t="s">
+      <c r="J2" s="67"/>
+      <c r="K2" s="67" t="s">
         <v>104</v>
       </c>
-      <c r="L2" s="62"/>
-      <c r="M2" s="72" t="s">
+      <c r="L2" s="67"/>
+      <c r="M2" s="77" t="s">
         <v>103</v>
       </c>
-      <c r="N2" s="68"/>
-      <c r="O2" s="62" t="s">
+      <c r="N2" s="73"/>
+      <c r="O2" s="67" t="s">
         <v>106</v>
       </c>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62" t="s">
+      <c r="P2" s="67"/>
+      <c r="Q2" s="67" t="s">
         <v>107</v>
       </c>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62" t="s">
+      <c r="R2" s="67"/>
+      <c r="S2" s="67" t="s">
         <v>100</v>
       </c>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62" t="s">
+      <c r="T2" s="67"/>
+      <c r="U2" s="67" t="s">
         <v>108</v>
       </c>
-      <c r="V2" s="72"/>
-      <c r="W2" s="75" t="s">
+      <c r="V2" s="77"/>
+      <c r="W2" s="80" t="s">
         <v>102</v>
       </c>
-      <c r="X2" s="76"/>
-      <c r="Y2" s="75" t="s">
+      <c r="X2" s="81"/>
+      <c r="Y2" s="80" t="s">
         <v>105</v>
       </c>
-      <c r="Z2" s="77"/>
-      <c r="AA2" s="78" t="s">
+      <c r="Z2" s="82"/>
+      <c r="AA2" s="83" t="s">
         <v>66</v>
       </c>
-      <c r="AB2" s="79"/>
-      <c r="AC2" s="68" t="s">
+      <c r="AB2" s="84"/>
+      <c r="AC2" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="AD2" s="62"/>
+      <c r="AD2" s="67"/>
     </row>
     <row r="3" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B3" s="32" t="s">
@@ -17548,34 +17663,34 @@
       </c>
     </row>
     <row r="32" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="F32" s="65" t="s">
+      <c r="F32" s="70" t="s">
         <v>56</v>
       </c>
-      <c r="G32" s="66"/>
-      <c r="H32" s="67"/>
-      <c r="I32" s="63">
+      <c r="G32" s="71"/>
+      <c r="H32" s="72"/>
+      <c r="I32" s="68">
         <f>C30+E30+G30+I30+K30+M30+O30+Q30+S30+U30+AA30+W30+Y30</f>
         <v>2648</v>
       </c>
-      <c r="J32" s="64"/>
+      <c r="J32" s="69"/>
     </row>
     <row r="33" spans="3:25" x14ac:dyDescent="0.3">
-      <c r="G33" s="70" t="s">
+      <c r="G33" s="75" t="s">
         <v>57</v>
       </c>
-      <c r="H33" s="70"/>
-      <c r="I33" s="63">
+      <c r="H33" s="75"/>
+      <c r="I33" s="68">
         <f>+D30+F30+H30+J30+L30+N30+P30+R30+T30+V30+AB30+X30+Z30</f>
         <v>1694.2299999999998</v>
       </c>
-      <c r="J33" s="64"/>
+      <c r="J33" s="69"/>
     </row>
     <row r="34" spans="3:25" x14ac:dyDescent="0.3">
-      <c r="I34" s="63">
+      <c r="I34" s="68">
         <f>I33-I32</f>
         <v>-953.77000000000021</v>
       </c>
-      <c r="J34" s="64"/>
+      <c r="J34" s="69"/>
       <c r="Y34">
         <f>2167+183+5*10</f>
         <v>2400</v>
@@ -17658,11 +17773,11 @@
         <v>64</v>
       </c>
       <c r="H39" s="42"/>
-      <c r="I39" s="71">
+      <c r="I39" s="76">
         <f>I37+I34</f>
         <v>1446.28</v>
       </c>
-      <c r="J39" s="71"/>
+      <c r="J39" s="76"/>
       <c r="M39" s="33"/>
     </row>
     <row r="41" spans="3:25" x14ac:dyDescent="0.3">
@@ -18949,70 +19064,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:38" ht="7.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="W1" s="73"/>
-      <c r="X1" s="74"/>
+      <c r="W1" s="78"/>
+      <c r="X1" s="79"/>
     </row>
     <row r="2" spans="2:38" ht="18" x14ac:dyDescent="0.35">
-      <c r="C2" s="62" t="s">
+      <c r="C2" s="67" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="62"/>
-      <c r="E2" s="72" t="s">
+      <c r="D2" s="67"/>
+      <c r="E2" s="77" t="s">
         <v>101</v>
       </c>
-      <c r="F2" s="68"/>
-      <c r="G2" s="62" t="s">
+      <c r="F2" s="73"/>
+      <c r="G2" s="67" t="s">
         <v>114</v>
       </c>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62" t="s">
+      <c r="H2" s="67"/>
+      <c r="I2" s="67" t="s">
         <v>115</v>
       </c>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62" t="s">
+      <c r="J2" s="67"/>
+      <c r="K2" s="67" t="s">
         <v>104</v>
       </c>
-      <c r="L2" s="62"/>
-      <c r="M2" s="72" t="s">
+      <c r="L2" s="67"/>
+      <c r="M2" s="77" t="s">
         <v>103</v>
       </c>
-      <c r="N2" s="68"/>
-      <c r="O2" s="62" t="s">
+      <c r="N2" s="73"/>
+      <c r="O2" s="67" t="s">
         <v>106</v>
       </c>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62" t="s">
+      <c r="P2" s="67"/>
+      <c r="Q2" s="67" t="s">
         <v>107</v>
       </c>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62" t="s">
+      <c r="R2" s="67"/>
+      <c r="S2" s="67" t="s">
         <v>100</v>
       </c>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62" t="s">
+      <c r="T2" s="67"/>
+      <c r="U2" s="67" t="s">
         <v>108</v>
       </c>
-      <c r="V2" s="72"/>
-      <c r="W2" s="75" t="s">
+      <c r="V2" s="77"/>
+      <c r="W2" s="80" t="s">
         <v>102</v>
       </c>
-      <c r="X2" s="76"/>
-      <c r="Y2" s="75" t="s">
+      <c r="X2" s="81"/>
+      <c r="Y2" s="80" t="s">
         <v>105</v>
       </c>
-      <c r="Z2" s="76"/>
-      <c r="AA2" s="80" t="s">
+      <c r="Z2" s="81"/>
+      <c r="AA2" s="85" t="s">
         <v>180</v>
       </c>
-      <c r="AB2" s="81"/>
-      <c r="AC2" s="78" t="s">
+      <c r="AB2" s="86"/>
+      <c r="AC2" s="83" t="s">
         <v>66</v>
       </c>
-      <c r="AD2" s="79"/>
-      <c r="AE2" s="68" t="s">
+      <c r="AD2" s="84"/>
+      <c r="AE2" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="AF2" s="62"/>
+      <c r="AF2" s="67"/>
     </row>
     <row r="3" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B3" s="32" t="s">
@@ -19117,51 +19232,103 @@
       <c r="B4" s="54" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="14"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="13"/>
-      <c r="S4" s="14"/>
-      <c r="T4" s="13"/>
-      <c r="U4" s="12"/>
-      <c r="V4" s="19"/>
-      <c r="W4" s="12"/>
-      <c r="X4" s="19"/>
-      <c r="Y4" s="12"/>
-      <c r="Z4" s="19"/>
-      <c r="AA4" s="12"/>
-      <c r="AB4" s="19"/>
+      <c r="C4" s="12">
+        <v>15</v>
+      </c>
+      <c r="D4" s="13">
+        <v>0</v>
+      </c>
+      <c r="E4" s="14">
+        <v>15</v>
+      </c>
+      <c r="F4" s="13">
+        <v>0</v>
+      </c>
+      <c r="G4" s="14">
+        <v>15</v>
+      </c>
+      <c r="H4" s="13">
+        <v>0</v>
+      </c>
+      <c r="I4" s="14">
+        <v>10</v>
+      </c>
+      <c r="J4" s="13">
+        <v>0</v>
+      </c>
+      <c r="K4" s="14">
+        <v>15</v>
+      </c>
+      <c r="L4" s="13">
+        <v>0</v>
+      </c>
+      <c r="M4" s="14">
+        <v>15</v>
+      </c>
+      <c r="N4" s="13">
+        <v>64</v>
+      </c>
+      <c r="O4" s="14">
+        <v>15</v>
+      </c>
+      <c r="P4" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="14">
+        <v>15</v>
+      </c>
+      <c r="R4" s="13">
+        <v>0</v>
+      </c>
+      <c r="S4" s="14">
+        <v>15</v>
+      </c>
+      <c r="T4" s="13">
+        <v>0</v>
+      </c>
+      <c r="U4" s="12">
+        <v>10</v>
+      </c>
+      <c r="V4" s="19">
+        <v>0</v>
+      </c>
+      <c r="W4" s="12">
+        <v>10</v>
+      </c>
+      <c r="X4" s="19">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="12">
+        <v>5</v>
+      </c>
+      <c r="Z4" s="19">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="12">
+        <v>15</v>
+      </c>
+      <c r="AB4" s="19">
+        <v>0</v>
+      </c>
       <c r="AC4" s="17">
         <f>U4+S4+Q4+O4+M4+K4+I4+G4+E4+C4+W4+Y4</f>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AD4" s="48">
         <f t="shared" ref="AD4" si="0">V4+T4+R4+P4+N4+L4+J4+H4+F4+D4</f>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AE4" s="1">
         <f>AC4</f>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF4" s="1">
         <f>AD4</f>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG4" s="1">
         <f>AF4-AE4</f>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH4" s="1"/>
     </row>
@@ -19205,17 +19372,23 @@
       </c>
       <c r="AE5" s="1">
         <f>AE4+AC5</f>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF5" s="1">
         <f>AF4+AD5</f>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG5" s="1">
         <f t="shared" ref="AG5:AG29" si="1">AF5-AE5</f>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH5" s="1"/>
+      <c r="AI5" s="87" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ5" s="87"/>
+      <c r="AK5" s="87"/>
+      <c r="AL5" s="87"/>
     </row>
     <row r="6" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B6" s="52" t="s">
@@ -19257,15 +19430,15 @@
       </c>
       <c r="AE6" s="1">
         <f t="shared" ref="AE6:AF21" si="3">AE5+AC6</f>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF6" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG6" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH6" s="1"/>
       <c r="AI6" s="43" t="s">
@@ -19321,22 +19494,22 @@
       </c>
       <c r="AE7" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF7" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG7" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH7" s="44" t="s">
         <v>71</v>
       </c>
       <c r="AI7" s="44">
         <f>+E30+'Punters 2024'!AE7</f>
-        <v>1208</v>
+        <v>1223</v>
       </c>
       <c r="AJ7" s="44">
         <f>+F30+'Punters 2024'!AF7</f>
@@ -19344,11 +19517,11 @@
       </c>
       <c r="AK7" s="49">
         <f>+AJ7-AI7</f>
-        <v>-665.4</v>
+        <v>-680.4</v>
       </c>
       <c r="AL7" s="47">
         <f>(AJ7-AI7)/AI7</f>
-        <v>-0.55082781456953644</v>
+        <v>-0.55633687653311525</v>
       </c>
     </row>
     <row r="8" spans="2:38" x14ac:dyDescent="0.3">
@@ -19391,22 +19564,22 @@
       </c>
       <c r="AE8" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF8" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG8" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH8" s="44" t="s">
         <v>72</v>
       </c>
       <c r="AI8" s="44">
         <f>+K30+'Punters 2024'!AE8</f>
-        <v>1388</v>
+        <v>1403</v>
       </c>
       <c r="AJ8" s="44">
         <f>+L30+'Punters 2024'!AF8</f>
@@ -19414,11 +19587,11 @@
       </c>
       <c r="AK8" s="50">
         <f t="shared" ref="AK8:AK18" si="4">+AJ8-AI8</f>
-        <v>-249.48000000000002</v>
+        <v>-264.48</v>
       </c>
       <c r="AL8" s="47">
         <f t="shared" ref="AL8:AL18" si="5">(AJ8-AI8)/AI8</f>
-        <v>-0.17974063400576371</v>
+        <v>-0.18851033499643621</v>
       </c>
     </row>
     <row r="9" spans="2:38" x14ac:dyDescent="0.3">
@@ -19461,22 +19634,22 @@
       </c>
       <c r="AE9" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF9" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG9" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH9" s="44" t="s">
         <v>73</v>
       </c>
       <c r="AI9" s="44">
         <f>+Y30+'Punters 2024'!AE9</f>
-        <v>1366.48</v>
+        <v>1371.48</v>
       </c>
       <c r="AJ9" s="44">
         <f>Z30+'Punters 2024'!AF9</f>
@@ -19484,11 +19657,11 @@
       </c>
       <c r="AK9" s="50">
         <f t="shared" si="4"/>
-        <v>-272.57999999999993</v>
+        <v>-277.57999999999993</v>
       </c>
       <c r="AL9" s="47">
         <f t="shared" si="5"/>
-        <v>-0.19947602599379421</v>
+        <v>-0.20239449353982553</v>
       </c>
     </row>
     <row r="10" spans="2:38" x14ac:dyDescent="0.3">
@@ -19531,22 +19704,22 @@
       </c>
       <c r="AE10" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF10" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG10" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH10" s="44" t="s">
         <v>74</v>
       </c>
       <c r="AI10" s="44">
         <f>+S30+'Punters 2024'!AE10</f>
-        <v>1364.9</v>
+        <v>1379.9</v>
       </c>
       <c r="AJ10" s="44">
         <f>+T30+'Punters 2024'!AF10</f>
@@ -19554,11 +19727,11 @@
       </c>
       <c r="AK10" s="50">
         <f t="shared" si="4"/>
-        <v>151.54999999999973</v>
+        <v>136.54999999999973</v>
       </c>
       <c r="AL10" s="45">
         <f t="shared" si="5"/>
-        <v>0.11103377536815863</v>
+        <v>9.8956446119283809E-2</v>
       </c>
     </row>
     <row r="11" spans="2:38" x14ac:dyDescent="0.3">
@@ -19601,34 +19774,34 @@
       </c>
       <c r="AE11" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF11" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG11" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH11" s="44" t="s">
         <v>75</v>
       </c>
       <c r="AI11" s="44">
         <f>+M30+'Punters 2024'!AE11</f>
-        <v>1073</v>
+        <v>1088</v>
       </c>
       <c r="AJ11" s="44">
         <f>+N30+'Punters 2024'!AF11</f>
-        <v>98.25</v>
+        <v>162.25</v>
       </c>
       <c r="AK11" s="49">
         <f t="shared" si="4"/>
-        <v>-974.75</v>
+        <v>-925.75</v>
       </c>
       <c r="AL11" s="47">
         <f t="shared" si="5"/>
-        <v>-0.9084342963653308</v>
+        <v>-0.85087316176470584</v>
       </c>
     </row>
     <row r="12" spans="2:38" x14ac:dyDescent="0.3">
@@ -19671,22 +19844,22 @@
       </c>
       <c r="AE12" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF12" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG12" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH12" s="44" t="s">
         <v>76</v>
       </c>
       <c r="AI12" s="44">
         <f>+U30+'Punters 2024'!AE12</f>
-        <v>1384.96</v>
+        <v>1394.96</v>
       </c>
       <c r="AJ12" s="44">
         <f>+V30+'Punters 2024'!AF12</f>
@@ -19694,11 +19867,11 @@
       </c>
       <c r="AK12" s="49">
         <f t="shared" si="4"/>
-        <v>-494.30000000000018</v>
+        <v>-504.30000000000018</v>
       </c>
       <c r="AL12" s="47">
         <f t="shared" si="5"/>
-        <v>-0.35690561460258791</v>
+        <v>-0.36151574238687861</v>
       </c>
     </row>
     <row r="13" spans="2:38" x14ac:dyDescent="0.3">
@@ -19741,22 +19914,22 @@
       </c>
       <c r="AE13" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF13" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG13" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH13" s="44" t="s">
         <v>77</v>
       </c>
       <c r="AI13" s="44">
         <f>+I30+'Punters 2024'!AE13</f>
-        <v>1346.3400000000001</v>
+        <v>1356.3400000000001</v>
       </c>
       <c r="AJ13" s="44">
         <f>+J30+'Punters 2024'!AF13</f>
@@ -19764,11 +19937,11 @@
       </c>
       <c r="AK13" s="49">
         <f t="shared" si="4"/>
-        <v>-720.10000000000014</v>
+        <v>-730.10000000000014</v>
       </c>
       <c r="AL13" s="47">
         <f t="shared" si="5"/>
-        <v>-0.5348574654247813</v>
+        <v>-0.53828686022678685</v>
       </c>
     </row>
     <row r="14" spans="2:38" x14ac:dyDescent="0.3">
@@ -19811,22 +19984,22 @@
       </c>
       <c r="AE14" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF14" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG14" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH14" s="44" t="s">
         <v>78</v>
       </c>
       <c r="AI14" s="44">
         <f>+Q30+'Punters 2024'!AE14</f>
-        <v>1353</v>
+        <v>1368</v>
       </c>
       <c r="AJ14" s="44">
         <f>+R30+'Punters 2024'!AF14</f>
@@ -19834,11 +20007,11 @@
       </c>
       <c r="AK14" s="49">
         <f t="shared" si="4"/>
-        <v>-715.53</v>
+        <v>-730.53</v>
       </c>
       <c r="AL14" s="47">
         <f t="shared" si="5"/>
-        <v>-0.52884700665188467</v>
+        <v>-0.5340131578947368</v>
       </c>
     </row>
     <row r="15" spans="2:38" x14ac:dyDescent="0.3">
@@ -19881,22 +20054,22 @@
       </c>
       <c r="AE15" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF15" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG15" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH15" s="44" t="s">
         <v>79</v>
       </c>
       <c r="AI15" s="44">
         <f>+O30+'Punters 2024'!AE15</f>
-        <v>1362.7</v>
+        <v>1377.7</v>
       </c>
       <c r="AJ15" s="44">
         <f>+P30+'Punters 2024'!AF15</f>
@@ -19904,11 +20077,11 @@
       </c>
       <c r="AK15" s="50">
         <f t="shared" si="4"/>
-        <v>333.38999999999987</v>
+        <v>318.38999999999987</v>
       </c>
       <c r="AL15" s="45">
         <f t="shared" si="5"/>
-        <v>0.24465399574374394</v>
+        <v>0.23110256224141676</v>
       </c>
     </row>
     <row r="16" spans="2:38" x14ac:dyDescent="0.3">
@@ -19951,22 +20124,22 @@
       </c>
       <c r="AE16" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF16" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG16" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH16" s="44" t="s">
         <v>80</v>
       </c>
       <c r="AI16" s="44">
         <f>+W30+'Punters 2024'!AE16</f>
-        <v>620</v>
+        <v>630</v>
       </c>
       <c r="AJ16" s="44">
         <f>+X30+'Punters 2024'!AF16</f>
@@ -19974,11 +20147,11 @@
       </c>
       <c r="AK16" s="49">
         <f t="shared" si="4"/>
-        <v>-468.75</v>
+        <v>-478.75</v>
       </c>
       <c r="AL16" s="47">
         <f t="shared" si="5"/>
-        <v>-0.75604838709677424</v>
+        <v>-0.75992063492063489</v>
       </c>
     </row>
     <row r="17" spans="2:38" x14ac:dyDescent="0.3">
@@ -20021,22 +20194,22 @@
       </c>
       <c r="AE17" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF17" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG17" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH17" s="44" t="s">
         <v>116</v>
       </c>
       <c r="AI17" s="44">
         <f>+C30</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="AJ17" s="44">
         <f>+D30</f>
@@ -20044,11 +20217,11 @@
       </c>
       <c r="AK17" s="49">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AL17" s="47" t="e">
+        <v>-15</v>
+      </c>
+      <c r="AL17" s="47">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="18" spans="2:38" x14ac:dyDescent="0.3">
@@ -20091,34 +20264,34 @@
       </c>
       <c r="AE18" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF18" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG18" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AH18" s="44" t="s">
+        <v>-91</v>
+      </c>
+      <c r="AH18" s="64" t="s">
         <v>117</v>
       </c>
-      <c r="AI18" s="44">
+      <c r="AI18" s="64">
         <f>+G30</f>
-        <v>0</v>
-      </c>
-      <c r="AJ18" s="44">
+        <v>15</v>
+      </c>
+      <c r="AJ18" s="64">
         <f>+H30</f>
         <v>0</v>
       </c>
-      <c r="AK18" s="49">
+      <c r="AK18" s="65">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AL18" s="47" t="e">
+        <v>-15</v>
+      </c>
+      <c r="AL18" s="66">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="19" spans="2:38" x14ac:dyDescent="0.3">
@@ -20161,17 +20334,23 @@
       </c>
       <c r="AE19" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF19" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG19" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AH19" s="1"/>
+        <v>-91</v>
+      </c>
+      <c r="AH19" s="62" t="s">
+        <v>182</v>
+      </c>
+      <c r="AI19" s="63"/>
+      <c r="AJ19" s="63"/>
+      <c r="AK19" s="63"/>
+      <c r="AL19" s="63"/>
     </row>
     <row r="20" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B20" s="53" t="s">
@@ -20213,15 +20392,15 @@
       </c>
       <c r="AE20" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF20" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG20" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH20" s="1"/>
     </row>
@@ -20265,15 +20444,15 @@
       </c>
       <c r="AE21" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF21" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG21" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH21" s="1"/>
     </row>
@@ -20317,15 +20496,15 @@
       </c>
       <c r="AE22" s="1">
         <f t="shared" ref="AE22:AF29" si="6">AE21+AC22</f>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF22" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG22" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH22" s="1"/>
     </row>
@@ -20369,15 +20548,15 @@
       </c>
       <c r="AE23" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF23" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG23" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH23" s="1"/>
     </row>
@@ -20421,15 +20600,15 @@
       </c>
       <c r="AE24" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF24" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG24" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH24" s="1"/>
     </row>
@@ -20473,15 +20652,15 @@
       </c>
       <c r="AE25" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF25" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG25" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH25" s="1"/>
     </row>
@@ -20525,15 +20704,15 @@
       </c>
       <c r="AE26" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF26" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG26" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH26" s="1"/>
     </row>
@@ -20577,15 +20756,15 @@
       </c>
       <c r="AE27" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF27" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG27" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH27" s="1"/>
     </row>
@@ -20629,15 +20808,15 @@
       </c>
       <c r="AE28" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF28" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG28" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH28" s="1"/>
     </row>
@@ -20681,15 +20860,15 @@
       </c>
       <c r="AE29" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AF29" s="1">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AG29" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-91</v>
       </c>
       <c r="AH29" s="1"/>
     </row>
@@ -20699,7 +20878,7 @@
       </c>
       <c r="C30" s="18">
         <f t="shared" ref="C30:AD30" si="8">SUM(C4:C29)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D30" s="18">
         <f t="shared" si="8"/>
@@ -20707,7 +20886,7 @@
       </c>
       <c r="E30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F30" s="18">
         <f t="shared" si="8"/>
@@ -20715,7 +20894,7 @@
       </c>
       <c r="G30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H30" s="18">
         <f t="shared" si="8"/>
@@ -20723,7 +20902,7 @@
       </c>
       <c r="I30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J30" s="18">
         <f t="shared" si="8"/>
@@ -20731,7 +20910,7 @@
       </c>
       <c r="K30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="L30" s="18">
         <f t="shared" si="8"/>
@@ -20739,15 +20918,15 @@
       </c>
       <c r="M30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="N30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="O30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="P30" s="18">
         <f t="shared" si="8"/>
@@ -20755,7 +20934,7 @@
       </c>
       <c r="Q30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="R30" s="18">
         <f t="shared" si="8"/>
@@ -20763,7 +20942,7 @@
       </c>
       <c r="S30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="T30" s="18">
         <f>SUM(T4:T29)</f>
@@ -20771,7 +20950,7 @@
       </c>
       <c r="U30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V30" s="21">
         <f t="shared" si="8"/>
@@ -20779,7 +20958,7 @@
       </c>
       <c r="W30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X30" s="21">
         <f t="shared" si="8"/>
@@ -20787,7 +20966,7 @@
       </c>
       <c r="Y30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Z30" s="21">
         <f t="shared" si="8"/>
@@ -20795,101 +20974,105 @@
       </c>
       <c r="AA30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="AB30" s="21">
-        <f t="shared" si="8"/>
+        <f>SUM(AB4:AB29)</f>
         <v>0</v>
       </c>
       <c r="AC30" s="29">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="AD30" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AE30" s="1"/>
     </row>
     <row r="31" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="D31" s="56" t="e">
+      <c r="D31" s="56">
         <f>(D30-C30)/C30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F31" s="34" t="e">
+        <v>-1</v>
+      </c>
+      <c r="F31" s="34">
         <f>(F30-E30)/E30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H31" s="34" t="e">
+        <v>-1</v>
+      </c>
+      <c r="H31" s="34">
         <f>(H30-G30)/G30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J31" s="34" t="e">
+        <v>-1</v>
+      </c>
+      <c r="J31" s="34">
         <f>(J30-I30)/I30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L31" s="28" t="e">
+        <v>-1</v>
+      </c>
+      <c r="L31" s="28">
         <f>(L30-K30)/K30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N31" s="28" t="e">
+        <v>-1</v>
+      </c>
+      <c r="N31" s="28">
         <f>(N30-M30)/M30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P31" s="28" t="e">
+        <v>3.2666666666666666</v>
+      </c>
+      <c r="P31" s="28">
         <f>(P30-O30)/O30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R31" s="28" t="e">
+        <v>-1</v>
+      </c>
+      <c r="R31" s="28">
         <f>(R30-Q30)/Q30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T31" s="22" t="e">
+        <v>-1</v>
+      </c>
+      <c r="T31" s="22">
         <f>(T30-S30)/S30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="V31" s="28" t="e">
+        <v>-1</v>
+      </c>
+      <c r="V31" s="28">
         <f>(V30-U30)/U30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X31" s="28" t="e">
+        <v>-1</v>
+      </c>
+      <c r="X31" s="28">
         <f>(X30-W30)/W30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z31" s="28" t="e">
+        <v>-1</v>
+      </c>
+      <c r="Z31" s="28">
         <f>(Z30-Y30)/Y30</f>
-        <v>#DIV/0!</v>
+        <v>-1</v>
+      </c>
+      <c r="AB31">
+        <f>(AB30-AA30)/AA30</f>
+        <v>-1</v>
       </c>
     </row>
     <row r="32" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="F32" s="65" t="s">
+      <c r="F32" s="70" t="s">
         <v>56</v>
       </c>
-      <c r="G32" s="66"/>
-      <c r="H32" s="67"/>
-      <c r="I32" s="63">
+      <c r="G32" s="71"/>
+      <c r="H32" s="72"/>
+      <c r="I32" s="68">
         <f>C30+E30+G30+I30+K30+M30+O30+Q30+S30+U30+AA30+W30+Y30</f>
-        <v>0</v>
-      </c>
-      <c r="J32" s="64"/>
+        <v>170</v>
+      </c>
+      <c r="J32" s="69"/>
     </row>
     <row r="33" spans="3:25" x14ac:dyDescent="0.3">
-      <c r="G33" s="70" t="s">
+      <c r="G33" s="75" t="s">
         <v>57</v>
       </c>
-      <c r="H33" s="70"/>
-      <c r="I33" s="63">
+      <c r="H33" s="75"/>
+      <c r="I33" s="68">
         <f>+D30+F30+H30+J30+L30+N30+P30+R30+T30+V30+AB30+X30+Z30</f>
-        <v>0</v>
-      </c>
-      <c r="J33" s="64"/>
+        <v>64</v>
+      </c>
+      <c r="J33" s="69"/>
     </row>
     <row r="34" spans="3:25" x14ac:dyDescent="0.3">
-      <c r="I34" s="63">
+      <c r="I34" s="68">
         <f>I33-I32</f>
-        <v>0</v>
-      </c>
-      <c r="J34" s="64"/>
+        <v>-106</v>
+      </c>
+      <c r="J34" s="69"/>
       <c r="Y34">
         <f>2167+183+5*10</f>
         <v>2400</v>
@@ -20898,7 +21081,7 @@
     <row r="35" spans="3:25" x14ac:dyDescent="0.3">
       <c r="C35" s="36">
         <f>C30+E30+G30+I30</f>
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="D35" s="36">
         <f>D30+F30+H30+J30</f>
@@ -20906,23 +21089,23 @@
       </c>
       <c r="E35" s="37">
         <f>D35-C35</f>
-        <v>0</v>
+        <v>-55</v>
       </c>
       <c r="I35" s="38">
         <f>O30+K30+M30+Q30</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="J35" s="38">
         <f>P30+L30+N30</f>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="K35" s="39">
         <f>J35-I35</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O35" s="40">
         <f>U30+W30+Y30+S30</f>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="P35" s="40">
         <f>V30+X30+T30+Z30</f>
@@ -20930,7 +21113,7 @@
       </c>
       <c r="Q35" s="41">
         <f>P35-O35</f>
-        <v>0</v>
+        <v>-40</v>
       </c>
       <c r="X35" s="55"/>
       <c r="Y35">
@@ -20940,21 +21123,21 @@
     </row>
     <row r="36" spans="3:25" x14ac:dyDescent="0.3">
       <c r="C36" s="36"/>
-      <c r="D36" s="34" t="e">
+      <c r="D36" s="34">
         <f>(D35-C35)/C35</f>
-        <v>#DIV/0!</v>
+        <v>-1</v>
       </c>
       <c r="E36" s="37"/>
       <c r="I36" s="38"/>
-      <c r="J36" s="34" t="e">
+      <c r="J36" s="34">
         <f>(J35-I35)/I35</f>
-        <v>#DIV/0!</v>
+        <v>6.6666666666666666E-2</v>
       </c>
       <c r="K36" s="39"/>
       <c r="O36" s="40"/>
-      <c r="P36" s="34" t="e">
+      <c r="P36" s="34">
         <f>(P35-O35)/O35</f>
-        <v>#DIV/0!</v>
+        <v>-1</v>
       </c>
       <c r="Q36" s="41"/>
       <c r="X36" s="55"/>
@@ -20972,11 +21155,11 @@
         <v>64</v>
       </c>
       <c r="H39" s="42"/>
-      <c r="I39" s="71">
+      <c r="I39" s="76">
         <f>I37+I34</f>
-        <v>2400.0500000000002</v>
-      </c>
-      <c r="J39" s="71"/>
+        <v>2294.0500000000002</v>
+      </c>
+      <c r="J39" s="76"/>
       <c r="M39" s="33"/>
     </row>
     <row r="41" spans="3:25" x14ac:dyDescent="0.3">
@@ -20985,7 +21168,7 @@
     <row r="43" spans="3:25" x14ac:dyDescent="0.3">
       <c r="C43" s="1">
         <f>C30+E30+G30+I30</f>
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="D43" s="1">
         <f>D30+F30+H30+J30</f>
@@ -20993,15 +21176,15 @@
       </c>
       <c r="I43" s="1">
         <f>O30+K30+M30</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J43" s="1">
         <f>P30+L30+N30</f>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="O43" s="1">
         <f>U30+Q30+S30</f>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="P43" s="1">
         <f>V30+R30+T30</f>
@@ -21011,20 +21194,20 @@
     <row r="44" spans="3:25" x14ac:dyDescent="0.3">
       <c r="D44" s="1">
         <f>D43-C43</f>
-        <v>0</v>
+        <v>-55</v>
       </c>
       <c r="J44" s="33">
         <f>J43-I43</f>
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="P44" s="33">
         <f>P43-O43</f>
-        <v>0</v>
+        <v>-40</v>
       </c>
     </row>
     <row r="46" spans="3:25" x14ac:dyDescent="0.3">
       <c r="V46" t="s">
-        <v>118</v>
+        <v>183</v>
       </c>
     </row>
     <row r="47" spans="3:25" x14ac:dyDescent="0.3">
@@ -21032,13 +21215,14 @@
         <v>88</v>
       </c>
       <c r="J47" t="s">
-        <v>119</v>
+        <v>184</v>
       </c>
       <c r="V47" t="s">
         <v>89</v>
       </c>
       <c r="W47">
-        <v>9</v>
+        <f>SUM('1 Leg Losses 2026'!G8)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="3:25" x14ac:dyDescent="0.3">
@@ -21058,7 +21242,8 @@
         <v>12</v>
       </c>
       <c r="W48">
-        <v>6</v>
+        <f>SUM('1 Leg Losses 2026'!G2)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="4:23" x14ac:dyDescent="0.3">
@@ -21079,7 +21264,8 @@
         <v>93</v>
       </c>
       <c r="W49">
-        <v>7</v>
+        <f>SUM('1 Leg Losses 2026'!G5)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="4:23" x14ac:dyDescent="0.3">
@@ -21100,7 +21286,8 @@
         <v>92</v>
       </c>
       <c r="W50">
-        <v>2</v>
+        <f>SUM('1 Leg Losses 2026'!G1)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="4:23" x14ac:dyDescent="0.3">
@@ -21121,7 +21308,8 @@
         <v>9</v>
       </c>
       <c r="W51">
-        <v>4</v>
+        <f>SUM('1 Leg Losses 2026'!G12)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="4:23" x14ac:dyDescent="0.3">
@@ -21142,7 +21330,8 @@
         <v>11</v>
       </c>
       <c r="W52">
-        <v>2</v>
+        <f>SUM('1 Leg Losses 2026'!G4)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="4:23" x14ac:dyDescent="0.3">
@@ -21163,7 +21352,8 @@
         <v>96</v>
       </c>
       <c r="W53">
-        <v>4</v>
+        <f>SUM('1 Leg Losses 2026'!G9)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="4:23" x14ac:dyDescent="0.3">
@@ -21184,7 +21374,8 @@
         <v>98</v>
       </c>
       <c r="W54">
-        <v>2</v>
+        <f>SUM('1 Leg Losses 2026'!G7)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="4:23" x14ac:dyDescent="0.3">
@@ -21193,7 +21384,7 @@
       </c>
       <c r="E55" s="1">
         <f>SUM(N30)</f>
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="J55" t="s">
         <v>98</v>
@@ -21205,7 +21396,8 @@
         <v>97</v>
       </c>
       <c r="W55">
-        <v>6</v>
+        <f>SUM('1 Leg Losses 2026'!G6)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="4:23" x14ac:dyDescent="0.3">
@@ -21226,7 +21418,8 @@
         <v>94</v>
       </c>
       <c r="W56">
-        <v>5</v>
+        <f>SUM('1 Leg Losses 2026'!G3)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="4:23" x14ac:dyDescent="0.3">
@@ -21247,7 +21440,8 @@
         <v>120</v>
       </c>
       <c r="W57">
-        <v>3</v>
+        <f>SUM('1 Leg Losses 2026'!G10)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="58" spans="4:23" x14ac:dyDescent="0.3">
@@ -21265,9 +21459,10 @@
         <v>0</v>
       </c>
       <c r="V58" t="s">
-        <v>121</v>
+        <v>185</v>
       </c>
       <c r="W58">
+        <f>SUM('1 Leg Losses 2026'!G13)</f>
         <v>1</v>
       </c>
     </row>
@@ -21286,38 +21481,44 @@
         <v>0</v>
       </c>
       <c r="V59" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="W59">
-        <f>SUM(W47:W58)</f>
-        <v>51</v>
+        <f>SUM('1 Leg Losses 2026'!G11)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="4:23" x14ac:dyDescent="0.3">
       <c r="D60" t="s">
-        <v>181</v>
+        <v>9</v>
       </c>
       <c r="E60" s="1">
-        <f>SUM(D30)</f>
+        <f>SUM(P30)</f>
         <v>0</v>
       </c>
       <c r="J60" t="s">
-        <v>181</v>
+        <v>9</v>
       </c>
       <c r="K60">
         <v>0</v>
+      </c>
+      <c r="V60" t="s">
+        <v>99</v>
+      </c>
+      <c r="W60">
+        <f>SUM(W47:W59)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="61" spans="4:23" x14ac:dyDescent="0.3">
       <c r="D61" t="s">
-        <v>9</v>
+        <v>185</v>
       </c>
       <c r="E61" s="1">
-        <f>SUM(P30)</f>
         <v>0</v>
       </c>
       <c r="J61" t="s">
-        <v>9</v>
+        <v>185</v>
       </c>
       <c r="K61">
         <v>0</v>
@@ -21328,19 +21529,20 @@
         <v>99</v>
       </c>
       <c r="E62" s="1">
-        <f>SUM(E49:E61)</f>
-        <v>0</v>
+        <f>SUM(E49:E60)</f>
+        <v>64</v>
       </c>
       <c r="J62" t="s">
         <v>99</v>
       </c>
       <c r="K62">
-        <f>SUM(K49:K61)</f>
+        <f>SUM(K49:K60)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="23">
+    <mergeCell ref="AI5:AL5"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="G2:H2"/>
@@ -21348,8 +21550,6 @@
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="AC2:AD2"/>
     <mergeCell ref="AE2:AF2"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:J32"/>
     <mergeCell ref="W1:X1"/>
     <mergeCell ref="M2:N2"/>
     <mergeCell ref="O2:P2"/>
@@ -21363,6 +21563,8 @@
     <mergeCell ref="U2:V2"/>
     <mergeCell ref="W2:X2"/>
     <mergeCell ref="Y2:Z2"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:J32"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="63" orientation="landscape"/>
@@ -21370,6 +21572,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="3e1ffae5-f160-4019-9720-1b11bf1b81a3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -21378,7 +21588,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002D8393059904904F9DB82DE4B9AFABF6" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f7bafc8adbaca2e93ffc3a1da3fd32d5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="3e1ffae5-f160-4019-9720-1b11bf1b81a3" xmlns:ns4="21753bd8-bffc-4cd2-a328-982ee854c895" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8f821f56a5d2247de677e71e73e5a99e" ns3:_="" ns4:_="">
     <xsd:import namespace="3e1ffae5-f160-4019-9720-1b11bf1b81a3"/>
@@ -21599,15 +21809,17 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="3e1ffae5-f160-4019-9720-1b11bf1b81a3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4D7A62A-0CB5-48B0-A73A-0A91BCC8EAEF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3e1ffae5-f160-4019-9720-1b11bf1b81a3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{948817D4-7F3F-493D-9D4C-B473DA03CC7E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -21615,7 +21827,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22BA772B-ABF0-4278-9CEF-D9160BBA9E07}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21634,18 +21846,8 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4D7A62A-0CB5-48B0-A73A-0A91BCC8EAEF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3e1ffae5-f160-4019-9720-1b11bf1b81a3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{0f7d30c2-cad0-4405-8153-25a6a3313da4}" enabled="1" method="Privileged" siteId="{6c637512-c417-4e78-9d62-b61258e4b619}" contentBits="0" removed="0"/>
+  <clbl:label id="{0f7d30c2-cad0-4405-8153-25a6a3313da4}" enabled="1" method="Privileged" siteId="{6c637512-c417-4e78-9d62-b61258e4b619}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>